<commit_message>
Corrections apportées suite aux revues c39fd4dba2e8e87bfc9851c371184162983f4202
</commit_message>
<xml_diff>
--- a/resolveIssues/ig/StructureDefinition-fr-encounter-care-document.xlsx
+++ b/resolveIssues/ig/StructureDefinition-fr-encounter-care-document.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4502" uniqueCount="659">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4358" uniqueCount="637">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-04T08:54:45+00:00</t>
+    <t>2026-06-04T14:47:37+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1370,73 +1370,13 @@
     <t>Type de participation</t>
   </si>
   <si>
-    <t>Encounter.participant:responsibleParty.type.id</t>
-  </si>
-  <si>
-    <t>Encounter.participant.type.id</t>
-  </si>
-  <si>
-    <t>Encounter.participant:responsibleParty.type.extension</t>
-  </si>
-  <si>
-    <t>Encounter.participant.type.extension</t>
-  </si>
-  <si>
-    <t>Encounter.participant:responsibleParty.type.coding</t>
-  </si>
-  <si>
-    <t>Encounter.participant.type.coding</t>
-  </si>
-  <si>
-    <t>Code defined by a terminology system</t>
-  </si>
-  <si>
-    <t>A reference to a code defined by a terminology system.</t>
-  </si>
-  <si>
-    <t>Codes may be defined very casually in enumerations, or code lists, up to very formal definitions such as SNOMED CT - see the HL7 v3 Core Principles for more information.  Ordering of codings is undefined and SHALL NOT be used to infer meaning. Generally, at most only one of the coding values will be labeled as UserSelected = true.</t>
-  </si>
-  <si>
-    <t>Allows for alternative encodings within a code system, and translations to other code systems.</t>
-  </si>
-  <si>
-    <t>https://interop.esante.gouv.fr/ig/document/core/ValueSet/fr-valueset-participation-type-encounter</t>
-  </si>
-  <si>
-    <t>CodeableConcept.coding</t>
-  </si>
-  <si>
-    <t>union(., ./translation)</t>
-  </si>
-  <si>
-    <t>C*E.1-8, C*E.10-22</t>
-  </si>
-  <si>
-    <t>Encounter.participant:responsibleParty.type.text</t>
-  </si>
-  <si>
-    <t>Encounter.participant.type.text</t>
-  </si>
-  <si>
-    <t>Plain text representation of the concept</t>
-  </si>
-  <si>
-    <t>A human language representation of the concept as seen/selected/uttered by the user who entered the data and/or which represents the intended meaning of the user.</t>
-  </si>
-  <si>
-    <t>Very often the text is the same as a displayName of one of the codings.</t>
-  </si>
-  <si>
-    <t>The codes from the terminologies do not always capture the correct meaning with all the nuances of the human using them, or sometimes there is no appropriate code at all. In these cases, the text is used to capture the full meaning of the source.</t>
-  </si>
-  <si>
-    <t>CodeableConcept.text</t>
-  </si>
-  <si>
-    <t>./originalText[mediaType/code="text/plain"]/data</t>
-  </si>
-  <si>
-    <t>C*E.9. But note many systems use C*E.2 for this</t>
+    <t>&lt;valueCodeableConcept xmlns="http://hl7.org/fhir"&gt;
+  &lt;coding&gt;
+    &lt;system value="https://mos.esante.gouv.fr/NOS/TRE_A13-HL7ParticipationType/FHIR/TRE-A13-HL7ParticipationType"/&gt;
+    &lt;code value="DIS"/&gt;
+    &lt;display value="Responsable de la sortie"/&gt;
+  &lt;/coding&gt;
+&lt;/valueCodeableConcept&gt;</t>
   </si>
   <si>
     <t>Encounter.participant:responsibleParty.period</t>
@@ -2350,7 +2290,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AN125"/>
+  <dimension ref="A1:AN121"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="49.73828125" customWidth="true" bestFit="true"/>
@@ -10017,7 +9957,7 @@
       </c>
       <c r="E68" s="2"/>
       <c r="F68" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G68" t="s" s="2">
         <v>79</v>
@@ -10052,7 +9992,7 @@
         <v>80</v>
       </c>
       <c r="S68" t="s" s="2">
-        <v>80</v>
+        <v>438</v>
       </c>
       <c r="T68" t="s" s="2">
         <v>80</v>
@@ -10120,10 +10060,10 @@
     </row>
     <row r="69">
       <c r="A69" t="s" s="2">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>439</v>
+        <v>417</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
@@ -10146,13 +10086,13 @@
         <v>80</v>
       </c>
       <c r="K69" t="s" s="2">
-        <v>102</v>
+        <v>254</v>
       </c>
       <c r="L69" t="s" s="2">
-        <v>103</v>
+        <v>418</v>
       </c>
       <c r="M69" t="s" s="2">
-        <v>104</v>
+        <v>419</v>
       </c>
       <c r="N69" s="2"/>
       <c r="O69" s="2"/>
@@ -10203,7 +10143,7 @@
         <v>80</v>
       </c>
       <c r="AF69" t="s" s="2">
-        <v>105</v>
+        <v>417</v>
       </c>
       <c r="AG69" t="s" s="2">
         <v>78</v>
@@ -10215,19 +10155,19 @@
         <v>80</v>
       </c>
       <c r="AJ69" t="s" s="2">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="AK69" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL69" t="s" s="2">
-        <v>106</v>
+        <v>420</v>
       </c>
       <c r="AM69" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN69" t="s" s="2">
-        <v>80</v>
+        <v>421</v>
       </c>
     </row>
     <row r="70">
@@ -10235,18 +10175,18 @@
         <v>440</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>441</v>
+        <v>422</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
-        <v>108</v>
+        <v>80</v>
       </c>
       <c r="E70" s="2"/>
       <c r="F70" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G70" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H70" t="s" s="2">
         <v>80</v>
@@ -10255,20 +10195,18 @@
         <v>80</v>
       </c>
       <c r="J70" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="K70" t="s" s="2">
-        <v>109</v>
+        <v>441</v>
       </c>
       <c r="L70" t="s" s="2">
-        <v>110</v>
+        <v>442</v>
       </c>
       <c r="M70" t="s" s="2">
-        <v>111</v>
-      </c>
-      <c r="N70" t="s" s="2">
-        <v>112</v>
-      </c>
+        <v>425</v>
+      </c>
+      <c r="N70" s="2"/>
       <c r="O70" s="2"/>
       <c r="P70" t="s" s="2">
         <v>80</v>
@@ -10305,53 +10243,55 @@
         <v>80</v>
       </c>
       <c r="AB70" t="s" s="2">
-        <v>113</v>
+        <v>80</v>
       </c>
       <c r="AC70" t="s" s="2">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="AD70" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE70" t="s" s="2">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="AF70" t="s" s="2">
-        <v>116</v>
+        <v>422</v>
       </c>
       <c r="AG70" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH70" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI70" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ70" t="s" s="2">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="AK70" t="s" s="2">
-        <v>80</v>
+        <v>426</v>
       </c>
       <c r="AL70" t="s" s="2">
-        <v>106</v>
+        <v>427</v>
       </c>
       <c r="AM70" t="s" s="2">
-        <v>80</v>
+        <v>428</v>
       </c>
       <c r="AN70" t="s" s="2">
-        <v>80</v>
+        <v>429</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s" s="2">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>443</v>
-      </c>
-      <c r="C71" s="2"/>
+        <v>399</v>
+      </c>
+      <c r="C71" t="s" s="2">
+        <v>444</v>
+      </c>
       <c r="D71" t="s" s="2">
         <v>80</v>
       </c>
@@ -10372,20 +10312,16 @@
         <v>89</v>
       </c>
       <c r="K71" t="s" s="2">
-        <v>146</v>
+        <v>279</v>
       </c>
       <c r="L71" t="s" s="2">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="M71" t="s" s="2">
-        <v>445</v>
-      </c>
-      <c r="N71" t="s" s="2">
-        <v>446</v>
-      </c>
-      <c r="O71" t="s" s="2">
-        <v>447</v>
-      </c>
+        <v>401</v>
+      </c>
+      <c r="N71" s="2"/>
+      <c r="O71" s="2"/>
       <c r="P71" t="s" s="2">
         <v>80</v>
       </c>
@@ -10409,11 +10345,13 @@
         <v>80</v>
       </c>
       <c r="X71" t="s" s="2">
-        <v>222</v>
-      </c>
-      <c r="Y71" s="2"/>
+        <v>80</v>
+      </c>
+      <c r="Y71" t="s" s="2">
+        <v>80</v>
+      </c>
       <c r="Z71" t="s" s="2">
-        <v>448</v>
+        <v>80</v>
       </c>
       <c r="AA71" t="s" s="2">
         <v>80</v>
@@ -10431,7 +10369,7 @@
         <v>80</v>
       </c>
       <c r="AF71" t="s" s="2">
-        <v>449</v>
+        <v>399</v>
       </c>
       <c r="AG71" t="s" s="2">
         <v>78</v>
@@ -10446,24 +10384,24 @@
         <v>100</v>
       </c>
       <c r="AK71" t="s" s="2">
-        <v>80</v>
+        <v>403</v>
       </c>
       <c r="AL71" t="s" s="2">
-        <v>450</v>
+        <v>404</v>
       </c>
       <c r="AM71" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN71" t="s" s="2">
-        <v>451</v>
+        <v>405</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="s" s="2">
-        <v>452</v>
+        <v>446</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>453</v>
+        <v>406</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
@@ -10483,23 +10421,19 @@
         <v>80</v>
       </c>
       <c r="J72" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="K72" t="s" s="2">
         <v>102</v>
       </c>
       <c r="L72" t="s" s="2">
-        <v>454</v>
+        <v>103</v>
       </c>
       <c r="M72" t="s" s="2">
-        <v>455</v>
-      </c>
-      <c r="N72" t="s" s="2">
-        <v>456</v>
-      </c>
-      <c r="O72" t="s" s="2">
-        <v>457</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="N72" s="2"/>
+      <c r="O72" s="2"/>
       <c r="P72" t="s" s="2">
         <v>80</v>
       </c>
@@ -10547,7 +10481,7 @@
         <v>80</v>
       </c>
       <c r="AF72" t="s" s="2">
-        <v>458</v>
+        <v>105</v>
       </c>
       <c r="AG72" t="s" s="2">
         <v>78</v>
@@ -10559,38 +10493,38 @@
         <v>80</v>
       </c>
       <c r="AJ72" t="s" s="2">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AK72" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL72" t="s" s="2">
-        <v>459</v>
+        <v>106</v>
       </c>
       <c r="AM72" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN72" t="s" s="2">
-        <v>460</v>
+        <v>80</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="s" s="2">
-        <v>461</v>
+        <v>447</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>417</v>
+        <v>407</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" t="s" s="2">
-        <v>80</v>
+        <v>108</v>
       </c>
       <c r="E73" s="2"/>
       <c r="F73" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G73" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H73" t="s" s="2">
         <v>80</v>
@@ -10602,15 +10536,17 @@
         <v>80</v>
       </c>
       <c r="K73" t="s" s="2">
-        <v>254</v>
+        <v>109</v>
       </c>
       <c r="L73" t="s" s="2">
-        <v>418</v>
+        <v>110</v>
       </c>
       <c r="M73" t="s" s="2">
-        <v>419</v>
-      </c>
-      <c r="N73" s="2"/>
+        <v>111</v>
+      </c>
+      <c r="N73" t="s" s="2">
+        <v>112</v>
+      </c>
       <c r="O73" s="2"/>
       <c r="P73" t="s" s="2">
         <v>80</v>
@@ -10659,71 +10595,75 @@
         <v>80</v>
       </c>
       <c r="AF73" t="s" s="2">
-        <v>417</v>
+        <v>116</v>
       </c>
       <c r="AG73" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH73" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI73" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ73" t="s" s="2">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="AK73" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL73" t="s" s="2">
-        <v>420</v>
+        <v>106</v>
       </c>
       <c r="AM73" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN73" t="s" s="2">
-        <v>421</v>
+        <v>80</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="s" s="2">
-        <v>462</v>
+        <v>448</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>422</v>
+        <v>408</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" t="s" s="2">
-        <v>80</v>
+        <v>286</v>
       </c>
       <c r="E74" s="2"/>
       <c r="F74" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="G74" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H74" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I74" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="J74" t="s" s="2">
         <v>89</v>
       </c>
       <c r="K74" t="s" s="2">
-        <v>463</v>
+        <v>109</v>
       </c>
       <c r="L74" t="s" s="2">
-        <v>464</v>
+        <v>287</v>
       </c>
       <c r="M74" t="s" s="2">
-        <v>425</v>
-      </c>
-      <c r="N74" s="2"/>
-      <c r="O74" s="2"/>
+        <v>288</v>
+      </c>
+      <c r="N74" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="O74" t="s" s="2">
+        <v>205</v>
+      </c>
       <c r="P74" t="s" s="2">
         <v>80</v>
       </c>
@@ -10771,43 +10711,41 @@
         <v>80</v>
       </c>
       <c r="AF74" t="s" s="2">
-        <v>422</v>
+        <v>289</v>
       </c>
       <c r="AG74" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH74" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI74" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ74" t="s" s="2">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="AK74" t="s" s="2">
-        <v>426</v>
+        <v>80</v>
       </c>
       <c r="AL74" t="s" s="2">
-        <v>427</v>
+        <v>191</v>
       </c>
       <c r="AM74" t="s" s="2">
-        <v>428</v>
+        <v>80</v>
       </c>
       <c r="AN74" t="s" s="2">
-        <v>429</v>
+        <v>80</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="s" s="2">
-        <v>465</v>
+        <v>449</v>
       </c>
       <c r="B75" t="s" s="2">
-        <v>399</v>
-      </c>
-      <c r="C75" t="s" s="2">
-        <v>466</v>
-      </c>
+        <v>409</v>
+      </c>
+      <c r="C75" s="2"/>
       <c r="D75" t="s" s="2">
         <v>80</v>
       </c>
@@ -10828,15 +10766,17 @@
         <v>89</v>
       </c>
       <c r="K75" t="s" s="2">
-        <v>279</v>
+        <v>228</v>
       </c>
       <c r="L75" t="s" s="2">
-        <v>467</v>
+        <v>437</v>
       </c>
       <c r="M75" t="s" s="2">
-        <v>401</v>
-      </c>
-      <c r="N75" s="2"/>
+        <v>411</v>
+      </c>
+      <c r="N75" t="s" s="2">
+        <v>412</v>
+      </c>
       <c r="O75" s="2"/>
       <c r="P75" t="s" s="2">
         <v>80</v>
@@ -10861,13 +10801,11 @@
         <v>80</v>
       </c>
       <c r="X75" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y75" t="s" s="2">
-        <v>80</v>
-      </c>
+        <v>222</v>
+      </c>
+      <c r="Y75" s="2"/>
       <c r="Z75" t="s" s="2">
-        <v>80</v>
+        <v>450</v>
       </c>
       <c r="AA75" t="s" s="2">
         <v>80</v>
@@ -10885,7 +10823,7 @@
         <v>80</v>
       </c>
       <c r="AF75" t="s" s="2">
-        <v>399</v>
+        <v>409</v>
       </c>
       <c r="AG75" t="s" s="2">
         <v>78</v>
@@ -10900,24 +10838,24 @@
         <v>100</v>
       </c>
       <c r="AK75" t="s" s="2">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="AL75" t="s" s="2">
-        <v>404</v>
+        <v>415</v>
       </c>
       <c r="AM75" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN75" t="s" s="2">
-        <v>405</v>
+        <v>416</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="s" s="2">
-        <v>468</v>
+        <v>451</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>406</v>
+        <v>417</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" t="s" s="2">
@@ -10940,13 +10878,13 @@
         <v>80</v>
       </c>
       <c r="K76" t="s" s="2">
-        <v>102</v>
+        <v>254</v>
       </c>
       <c r="L76" t="s" s="2">
-        <v>103</v>
+        <v>418</v>
       </c>
       <c r="M76" t="s" s="2">
-        <v>104</v>
+        <v>419</v>
       </c>
       <c r="N76" s="2"/>
       <c r="O76" s="2"/>
@@ -10997,7 +10935,7 @@
         <v>80</v>
       </c>
       <c r="AF76" t="s" s="2">
-        <v>105</v>
+        <v>417</v>
       </c>
       <c r="AG76" t="s" s="2">
         <v>78</v>
@@ -11009,38 +10947,38 @@
         <v>80</v>
       </c>
       <c r="AJ76" t="s" s="2">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="AK76" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL76" t="s" s="2">
-        <v>106</v>
+        <v>420</v>
       </c>
       <c r="AM76" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN76" t="s" s="2">
-        <v>80</v>
+        <v>421</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="s" s="2">
-        <v>469</v>
+        <v>452</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>407</v>
+        <v>422</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" t="s" s="2">
-        <v>108</v>
+        <v>80</v>
       </c>
       <c r="E77" s="2"/>
       <c r="F77" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G77" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H77" t="s" s="2">
         <v>80</v>
@@ -11049,20 +10987,18 @@
         <v>80</v>
       </c>
       <c r="J77" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="K77" t="s" s="2">
-        <v>109</v>
+        <v>441</v>
       </c>
       <c r="L77" t="s" s="2">
-        <v>110</v>
+        <v>453</v>
       </c>
       <c r="M77" t="s" s="2">
-        <v>111</v>
-      </c>
-      <c r="N77" t="s" s="2">
-        <v>112</v>
-      </c>
+        <v>425</v>
+      </c>
+      <c r="N77" s="2"/>
       <c r="O77" s="2"/>
       <c r="P77" t="s" s="2">
         <v>80</v>
@@ -11111,43 +11047,43 @@
         <v>80</v>
       </c>
       <c r="AF77" t="s" s="2">
-        <v>116</v>
+        <v>422</v>
       </c>
       <c r="AG77" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH77" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI77" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ77" t="s" s="2">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="AK77" t="s" s="2">
-        <v>80</v>
+        <v>426</v>
       </c>
       <c r="AL77" t="s" s="2">
-        <v>106</v>
+        <v>427</v>
       </c>
       <c r="AM77" t="s" s="2">
-        <v>80</v>
+        <v>428</v>
       </c>
       <c r="AN77" t="s" s="2">
-        <v>80</v>
+        <v>429</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="s" s="2">
-        <v>470</v>
+        <v>454</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>408</v>
+        <v>454</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" t="s" s="2">
-        <v>286</v>
+        <v>80</v>
       </c>
       <c r="E78" s="2"/>
       <c r="F78" t="s" s="2">
@@ -11160,26 +11096,22 @@
         <v>80</v>
       </c>
       <c r="I78" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="J78" t="s" s="2">
         <v>89</v>
       </c>
       <c r="K78" t="s" s="2">
-        <v>109</v>
+        <v>455</v>
       </c>
       <c r="L78" t="s" s="2">
-        <v>287</v>
+        <v>456</v>
       </c>
       <c r="M78" t="s" s="2">
-        <v>288</v>
-      </c>
-      <c r="N78" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="O78" t="s" s="2">
-        <v>205</v>
-      </c>
+        <v>457</v>
+      </c>
+      <c r="N78" s="2"/>
+      <c r="O78" s="2"/>
       <c r="P78" t="s" s="2">
         <v>80</v>
       </c>
@@ -11227,7 +11159,7 @@
         <v>80</v>
       </c>
       <c r="AF78" t="s" s="2">
-        <v>289</v>
+        <v>454</v>
       </c>
       <c r="AG78" t="s" s="2">
         <v>78</v>
@@ -11239,27 +11171,27 @@
         <v>80</v>
       </c>
       <c r="AJ78" t="s" s="2">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="AK78" t="s" s="2">
-        <v>80</v>
+        <v>397</v>
       </c>
       <c r="AL78" t="s" s="2">
-        <v>191</v>
+        <v>458</v>
       </c>
       <c r="AM78" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN78" t="s" s="2">
-        <v>80</v>
+        <v>459</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="s" s="2">
-        <v>471</v>
+        <v>460</v>
       </c>
       <c r="B79" t="s" s="2">
-        <v>409</v>
+        <v>460</v>
       </c>
       <c r="C79" s="2"/>
       <c r="D79" t="s" s="2">
@@ -11267,10 +11199,10 @@
       </c>
       <c r="E79" s="2"/>
       <c r="F79" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G79" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H79" t="s" s="2">
         <v>80</v>
@@ -11279,19 +11211,19 @@
         <v>80</v>
       </c>
       <c r="J79" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="K79" t="s" s="2">
-        <v>228</v>
+        <v>254</v>
       </c>
       <c r="L79" t="s" s="2">
-        <v>437</v>
+        <v>461</v>
       </c>
       <c r="M79" t="s" s="2">
-        <v>411</v>
+        <v>462</v>
       </c>
       <c r="N79" t="s" s="2">
-        <v>412</v>
+        <v>463</v>
       </c>
       <c r="O79" s="2"/>
       <c r="P79" t="s" s="2">
@@ -11317,11 +11249,13 @@
         <v>80</v>
       </c>
       <c r="X79" t="s" s="2">
-        <v>222</v>
-      </c>
-      <c r="Y79" s="2"/>
+        <v>80</v>
+      </c>
+      <c r="Y79" t="s" s="2">
+        <v>80</v>
+      </c>
       <c r="Z79" t="s" s="2">
-        <v>472</v>
+        <v>80</v>
       </c>
       <c r="AA79" t="s" s="2">
         <v>80</v>
@@ -11339,13 +11273,13 @@
         <v>80</v>
       </c>
       <c r="AF79" t="s" s="2">
-        <v>409</v>
+        <v>460</v>
       </c>
       <c r="AG79" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH79" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI79" t="s" s="2">
         <v>80</v>
@@ -11354,24 +11288,24 @@
         <v>100</v>
       </c>
       <c r="AK79" t="s" s="2">
-        <v>414</v>
+        <v>464</v>
       </c>
       <c r="AL79" t="s" s="2">
-        <v>415</v>
+        <v>465</v>
       </c>
       <c r="AM79" t="s" s="2">
-        <v>80</v>
+        <v>466</v>
       </c>
       <c r="AN79" t="s" s="2">
-        <v>416</v>
+        <v>467</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="s" s="2">
-        <v>473</v>
+        <v>468</v>
       </c>
       <c r="B80" t="s" s="2">
-        <v>417</v>
+        <v>468</v>
       </c>
       <c r="C80" s="2"/>
       <c r="D80" t="s" s="2">
@@ -11394,15 +11328,17 @@
         <v>80</v>
       </c>
       <c r="K80" t="s" s="2">
-        <v>254</v>
+        <v>469</v>
       </c>
       <c r="L80" t="s" s="2">
-        <v>418</v>
+        <v>470</v>
       </c>
       <c r="M80" t="s" s="2">
-        <v>419</v>
-      </c>
-      <c r="N80" s="2"/>
+        <v>471</v>
+      </c>
+      <c r="N80" t="s" s="2">
+        <v>472</v>
+      </c>
       <c r="O80" s="2"/>
       <c r="P80" t="s" s="2">
         <v>80</v>
@@ -11451,7 +11387,7 @@
         <v>80</v>
       </c>
       <c r="AF80" t="s" s="2">
-        <v>417</v>
+        <v>468</v>
       </c>
       <c r="AG80" t="s" s="2">
         <v>78</v>
@@ -11466,35 +11402,35 @@
         <v>100</v>
       </c>
       <c r="AK80" t="s" s="2">
-        <v>80</v>
+        <v>464</v>
       </c>
       <c r="AL80" t="s" s="2">
-        <v>420</v>
+        <v>473</v>
       </c>
       <c r="AM80" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN80" t="s" s="2">
-        <v>421</v>
+        <v>474</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s" s="2">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B81" t="s" s="2">
-        <v>422</v>
+        <v>475</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
-        <v>80</v>
+        <v>476</v>
       </c>
       <c r="E81" s="2"/>
       <c r="F81" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="G81" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H81" t="s" s="2">
         <v>80</v>
@@ -11506,15 +11442,17 @@
         <v>89</v>
       </c>
       <c r="K81" t="s" s="2">
-        <v>463</v>
+        <v>228</v>
       </c>
       <c r="L81" t="s" s="2">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="M81" t="s" s="2">
-        <v>425</v>
-      </c>
-      <c r="N81" s="2"/>
+        <v>478</v>
+      </c>
+      <c r="N81" t="s" s="2">
+        <v>479</v>
+      </c>
       <c r="O81" s="2"/>
       <c r="P81" t="s" s="2">
         <v>80</v>
@@ -11539,13 +11477,13 @@
         <v>80</v>
       </c>
       <c r="X81" t="s" s="2">
-        <v>80</v>
+        <v>172</v>
       </c>
       <c r="Y81" t="s" s="2">
-        <v>80</v>
+        <v>480</v>
       </c>
       <c r="Z81" t="s" s="2">
-        <v>80</v>
+        <v>481</v>
       </c>
       <c r="AA81" t="s" s="2">
         <v>80</v>
@@ -11563,13 +11501,13 @@
         <v>80</v>
       </c>
       <c r="AF81" t="s" s="2">
-        <v>422</v>
+        <v>475</v>
       </c>
       <c r="AG81" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH81" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI81" t="s" s="2">
         <v>80</v>
@@ -11578,28 +11516,28 @@
         <v>100</v>
       </c>
       <c r="AK81" t="s" s="2">
-        <v>426</v>
+        <v>482</v>
       </c>
       <c r="AL81" t="s" s="2">
-        <v>427</v>
+        <v>483</v>
       </c>
       <c r="AM81" t="s" s="2">
-        <v>428</v>
+        <v>484</v>
       </c>
       <c r="AN81" t="s" s="2">
-        <v>429</v>
+        <v>485</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="s" s="2">
-        <v>476</v>
+        <v>486</v>
       </c>
       <c r="B82" t="s" s="2">
-        <v>476</v>
+        <v>486</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" t="s" s="2">
-        <v>80</v>
+        <v>476</v>
       </c>
       <c r="E82" s="2"/>
       <c r="F82" t="s" s="2">
@@ -11618,15 +11556,17 @@
         <v>89</v>
       </c>
       <c r="K82" t="s" s="2">
-        <v>477</v>
+        <v>487</v>
       </c>
       <c r="L82" t="s" s="2">
+        <v>488</v>
+      </c>
+      <c r="M82" t="s" s="2">
         <v>478</v>
       </c>
-      <c r="M82" t="s" s="2">
+      <c r="N82" t="s" s="2">
         <v>479</v>
       </c>
-      <c r="N82" s="2"/>
       <c r="O82" s="2"/>
       <c r="P82" t="s" s="2">
         <v>80</v>
@@ -11675,7 +11615,7 @@
         <v>80</v>
       </c>
       <c r="AF82" t="s" s="2">
-        <v>476</v>
+        <v>486</v>
       </c>
       <c r="AG82" t="s" s="2">
         <v>78</v>
@@ -11690,24 +11630,24 @@
         <v>100</v>
       </c>
       <c r="AK82" t="s" s="2">
-        <v>397</v>
+        <v>482</v>
       </c>
       <c r="AL82" t="s" s="2">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="AM82" t="s" s="2">
-        <v>80</v>
+        <v>484</v>
       </c>
       <c r="AN82" t="s" s="2">
-        <v>481</v>
+        <v>485</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="s" s="2">
-        <v>482</v>
+        <v>489</v>
       </c>
       <c r="B83" t="s" s="2">
-        <v>482</v>
+        <v>489</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
@@ -11715,10 +11655,10 @@
       </c>
       <c r="E83" s="2"/>
       <c r="F83" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="G83" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H83" t="s" s="2">
         <v>80</v>
@@ -11727,20 +11667,18 @@
         <v>80</v>
       </c>
       <c r="J83" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="K83" t="s" s="2">
-        <v>254</v>
+        <v>279</v>
       </c>
       <c r="L83" t="s" s="2">
-        <v>483</v>
+        <v>490</v>
       </c>
       <c r="M83" t="s" s="2">
-        <v>484</v>
-      </c>
-      <c r="N83" t="s" s="2">
-        <v>485</v>
-      </c>
+        <v>491</v>
+      </c>
+      <c r="N83" s="2"/>
       <c r="O83" s="2"/>
       <c r="P83" t="s" s="2">
         <v>80</v>
@@ -11789,13 +11727,13 @@
         <v>80</v>
       </c>
       <c r="AF83" t="s" s="2">
-        <v>482</v>
+        <v>489</v>
       </c>
       <c r="AG83" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH83" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI83" t="s" s="2">
         <v>80</v>
@@ -11804,24 +11742,24 @@
         <v>100</v>
       </c>
       <c r="AK83" t="s" s="2">
-        <v>486</v>
+        <v>80</v>
       </c>
       <c r="AL83" t="s" s="2">
-        <v>487</v>
+        <v>492</v>
       </c>
       <c r="AM83" t="s" s="2">
-        <v>488</v>
+        <v>80</v>
       </c>
       <c r="AN83" t="s" s="2">
-        <v>489</v>
+        <v>80</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="s" s="2">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="B84" t="s" s="2">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" t="s" s="2">
@@ -11844,17 +11782,15 @@
         <v>80</v>
       </c>
       <c r="K84" t="s" s="2">
-        <v>491</v>
+        <v>102</v>
       </c>
       <c r="L84" t="s" s="2">
-        <v>492</v>
+        <v>103</v>
       </c>
       <c r="M84" t="s" s="2">
-        <v>493</v>
-      </c>
-      <c r="N84" t="s" s="2">
-        <v>494</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="N84" s="2"/>
       <c r="O84" s="2"/>
       <c r="P84" t="s" s="2">
         <v>80</v>
@@ -11903,7 +11839,7 @@
         <v>80</v>
       </c>
       <c r="AF84" t="s" s="2">
-        <v>490</v>
+        <v>105</v>
       </c>
       <c r="AG84" t="s" s="2">
         <v>78</v>
@@ -11915,31 +11851,31 @@
         <v>80</v>
       </c>
       <c r="AJ84" t="s" s="2">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AK84" t="s" s="2">
-        <v>486</v>
+        <v>80</v>
       </c>
       <c r="AL84" t="s" s="2">
-        <v>495</v>
+        <v>106</v>
       </c>
       <c r="AM84" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN84" t="s" s="2">
-        <v>496</v>
+        <v>80</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="s" s="2">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="B85" t="s" s="2">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" t="s" s="2">
-        <v>498</v>
+        <v>108</v>
       </c>
       <c r="E85" s="2"/>
       <c r="F85" t="s" s="2">
@@ -11955,19 +11891,19 @@
         <v>80</v>
       </c>
       <c r="J85" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="K85" t="s" s="2">
-        <v>228</v>
+        <v>109</v>
       </c>
       <c r="L85" t="s" s="2">
-        <v>499</v>
+        <v>110</v>
       </c>
       <c r="M85" t="s" s="2">
-        <v>500</v>
+        <v>111</v>
       </c>
       <c r="N85" t="s" s="2">
-        <v>501</v>
+        <v>112</v>
       </c>
       <c r="O85" s="2"/>
       <c r="P85" t="s" s="2">
@@ -11993,13 +11929,13 @@
         <v>80</v>
       </c>
       <c r="X85" t="s" s="2">
-        <v>172</v>
+        <v>80</v>
       </c>
       <c r="Y85" t="s" s="2">
-        <v>502</v>
+        <v>80</v>
       </c>
       <c r="Z85" t="s" s="2">
-        <v>503</v>
+        <v>80</v>
       </c>
       <c r="AA85" t="s" s="2">
         <v>80</v>
@@ -12017,7 +11953,7 @@
         <v>80</v>
       </c>
       <c r="AF85" t="s" s="2">
-        <v>497</v>
+        <v>116</v>
       </c>
       <c r="AG85" t="s" s="2">
         <v>78</v>
@@ -12029,31 +11965,31 @@
         <v>80</v>
       </c>
       <c r="AJ85" t="s" s="2">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="AK85" t="s" s="2">
-        <v>504</v>
+        <v>80</v>
       </c>
       <c r="AL85" t="s" s="2">
-        <v>505</v>
+        <v>106</v>
       </c>
       <c r="AM85" t="s" s="2">
-        <v>506</v>
+        <v>80</v>
       </c>
       <c r="AN85" t="s" s="2">
-        <v>507</v>
+        <v>80</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="s" s="2">
-        <v>508</v>
+        <v>495</v>
       </c>
       <c r="B86" t="s" s="2">
-        <v>508</v>
+        <v>495</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
-        <v>498</v>
+        <v>286</v>
       </c>
       <c r="E86" s="2"/>
       <c r="F86" t="s" s="2">
@@ -12066,24 +12002,26 @@
         <v>80</v>
       </c>
       <c r="I86" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="J86" t="s" s="2">
         <v>89</v>
       </c>
       <c r="K86" t="s" s="2">
-        <v>509</v>
+        <v>109</v>
       </c>
       <c r="L86" t="s" s="2">
-        <v>510</v>
+        <v>287</v>
       </c>
       <c r="M86" t="s" s="2">
-        <v>500</v>
+        <v>288</v>
       </c>
       <c r="N86" t="s" s="2">
-        <v>501</v>
-      </c>
-      <c r="O86" s="2"/>
+        <v>112</v>
+      </c>
+      <c r="O86" t="s" s="2">
+        <v>205</v>
+      </c>
       <c r="P86" t="s" s="2">
         <v>80</v>
       </c>
@@ -12131,7 +12069,7 @@
         <v>80</v>
       </c>
       <c r="AF86" t="s" s="2">
-        <v>508</v>
+        <v>289</v>
       </c>
       <c r="AG86" t="s" s="2">
         <v>78</v>
@@ -12143,38 +12081,38 @@
         <v>80</v>
       </c>
       <c r="AJ86" t="s" s="2">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="AK86" t="s" s="2">
-        <v>504</v>
+        <v>80</v>
       </c>
       <c r="AL86" t="s" s="2">
-        <v>505</v>
+        <v>191</v>
       </c>
       <c r="AM86" t="s" s="2">
-        <v>506</v>
+        <v>80</v>
       </c>
       <c r="AN86" t="s" s="2">
-        <v>507</v>
+        <v>80</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="s" s="2">
-        <v>511</v>
+        <v>496</v>
       </c>
       <c r="B87" t="s" s="2">
-        <v>511</v>
+        <v>496</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
-        <v>80</v>
+        <v>497</v>
       </c>
       <c r="E87" s="2"/>
       <c r="F87" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G87" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H87" t="s" s="2">
         <v>80</v>
@@ -12186,15 +12124,17 @@
         <v>89</v>
       </c>
       <c r="K87" t="s" s="2">
-        <v>279</v>
+        <v>498</v>
       </c>
       <c r="L87" t="s" s="2">
-        <v>512</v>
+        <v>499</v>
       </c>
       <c r="M87" t="s" s="2">
-        <v>513</v>
-      </c>
-      <c r="N87" s="2"/>
+        <v>500</v>
+      </c>
+      <c r="N87" t="s" s="2">
+        <v>479</v>
+      </c>
       <c r="O87" s="2"/>
       <c r="P87" t="s" s="2">
         <v>80</v>
@@ -12243,13 +12183,13 @@
         <v>80</v>
       </c>
       <c r="AF87" t="s" s="2">
-        <v>511</v>
+        <v>496</v>
       </c>
       <c r="AG87" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="AH87" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI87" t="s" s="2">
         <v>80</v>
@@ -12258,24 +12198,24 @@
         <v>100</v>
       </c>
       <c r="AK87" t="s" s="2">
-        <v>80</v>
+        <v>501</v>
       </c>
       <c r="AL87" t="s" s="2">
-        <v>514</v>
+        <v>502</v>
       </c>
       <c r="AM87" t="s" s="2">
-        <v>80</v>
+        <v>484</v>
       </c>
       <c r="AN87" t="s" s="2">
-        <v>80</v>
+        <v>503</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="s" s="2">
-        <v>515</v>
+        <v>504</v>
       </c>
       <c r="B88" t="s" s="2">
-        <v>515</v>
+        <v>504</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
@@ -12298,13 +12238,13 @@
         <v>80</v>
       </c>
       <c r="K88" t="s" s="2">
-        <v>102</v>
+        <v>228</v>
       </c>
       <c r="L88" t="s" s="2">
-        <v>103</v>
+        <v>505</v>
       </c>
       <c r="M88" t="s" s="2">
-        <v>104</v>
+        <v>506</v>
       </c>
       <c r="N88" s="2"/>
       <c r="O88" s="2"/>
@@ -12331,13 +12271,13 @@
         <v>80</v>
       </c>
       <c r="X88" t="s" s="2">
-        <v>80</v>
+        <v>172</v>
       </c>
       <c r="Y88" t="s" s="2">
-        <v>80</v>
+        <v>507</v>
       </c>
       <c r="Z88" t="s" s="2">
-        <v>80</v>
+        <v>508</v>
       </c>
       <c r="AA88" t="s" s="2">
         <v>80</v>
@@ -12355,7 +12295,7 @@
         <v>80</v>
       </c>
       <c r="AF88" t="s" s="2">
-        <v>105</v>
+        <v>504</v>
       </c>
       <c r="AG88" t="s" s="2">
         <v>78</v>
@@ -12367,7 +12307,7 @@
         <v>80</v>
       </c>
       <c r="AJ88" t="s" s="2">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="AK88" t="s" s="2">
         <v>80</v>
@@ -12384,21 +12324,21 @@
     </row>
     <row r="89">
       <c r="A89" t="s" s="2">
-        <v>516</v>
+        <v>509</v>
       </c>
       <c r="B89" t="s" s="2">
-        <v>516</v>
+        <v>509</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
-        <v>108</v>
+        <v>80</v>
       </c>
       <c r="E89" s="2"/>
       <c r="F89" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G89" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H89" t="s" s="2">
         <v>80</v>
@@ -12410,17 +12350,15 @@
         <v>80</v>
       </c>
       <c r="K89" t="s" s="2">
-        <v>109</v>
+        <v>510</v>
       </c>
       <c r="L89" t="s" s="2">
-        <v>110</v>
+        <v>511</v>
       </c>
       <c r="M89" t="s" s="2">
-        <v>111</v>
-      </c>
-      <c r="N89" t="s" s="2">
-        <v>112</v>
-      </c>
+        <v>512</v>
+      </c>
+      <c r="N89" s="2"/>
       <c r="O89" s="2"/>
       <c r="P89" t="s" s="2">
         <v>80</v>
@@ -12469,25 +12407,25 @@
         <v>80</v>
       </c>
       <c r="AF89" t="s" s="2">
-        <v>116</v>
+        <v>509</v>
       </c>
       <c r="AG89" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH89" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI89" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ89" t="s" s="2">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="AK89" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL89" t="s" s="2">
-        <v>106</v>
+        <v>513</v>
       </c>
       <c r="AM89" t="s" s="2">
         <v>80</v>
@@ -12498,46 +12436,44 @@
     </row>
     <row r="90">
       <c r="A90" t="s" s="2">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="B90" t="s" s="2">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="C90" s="2"/>
       <c r="D90" t="s" s="2">
-        <v>286</v>
+        <v>80</v>
       </c>
       <c r="E90" s="2"/>
       <c r="F90" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G90" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H90" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I90" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="J90" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="K90" t="s" s="2">
-        <v>109</v>
+        <v>515</v>
       </c>
       <c r="L90" t="s" s="2">
-        <v>287</v>
+        <v>516</v>
       </c>
       <c r="M90" t="s" s="2">
-        <v>288</v>
+        <v>517</v>
       </c>
       <c r="N90" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="O90" t="s" s="2">
-        <v>205</v>
-      </c>
+        <v>518</v>
+      </c>
+      <c r="O90" s="2"/>
       <c r="P90" t="s" s="2">
         <v>80</v>
       </c>
@@ -12585,7 +12521,7 @@
         <v>80</v>
       </c>
       <c r="AF90" t="s" s="2">
-        <v>289</v>
+        <v>514</v>
       </c>
       <c r="AG90" t="s" s="2">
         <v>78</v>
@@ -12597,13 +12533,13 @@
         <v>80</v>
       </c>
       <c r="AJ90" t="s" s="2">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="AK90" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL90" t="s" s="2">
-        <v>191</v>
+        <v>519</v>
       </c>
       <c r="AM90" t="s" s="2">
         <v>80</v>
@@ -12614,18 +12550,18 @@
     </row>
     <row r="91">
       <c r="A91" t="s" s="2">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B91" t="s" s="2">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="C91" s="2"/>
       <c r="D91" t="s" s="2">
-        <v>519</v>
+        <v>80</v>
       </c>
       <c r="E91" s="2"/>
       <c r="F91" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="G91" t="s" s="2">
         <v>88</v>
@@ -12637,10 +12573,10 @@
         <v>80</v>
       </c>
       <c r="J91" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="K91" t="s" s="2">
-        <v>520</v>
+        <v>279</v>
       </c>
       <c r="L91" t="s" s="2">
         <v>521</v>
@@ -12649,7 +12585,7 @@
         <v>522</v>
       </c>
       <c r="N91" t="s" s="2">
-        <v>501</v>
+        <v>523</v>
       </c>
       <c r="O91" s="2"/>
       <c r="P91" t="s" s="2">
@@ -12699,10 +12635,10 @@
         <v>80</v>
       </c>
       <c r="AF91" t="s" s="2">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="AG91" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="AH91" t="s" s="2">
         <v>88</v>
@@ -12714,24 +12650,24 @@
         <v>100</v>
       </c>
       <c r="AK91" t="s" s="2">
-        <v>523</v>
+        <v>80</v>
       </c>
       <c r="AL91" t="s" s="2">
         <v>524</v>
       </c>
       <c r="AM91" t="s" s="2">
-        <v>506</v>
+        <v>80</v>
       </c>
       <c r="AN91" t="s" s="2">
-        <v>525</v>
+        <v>80</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="s" s="2">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="B92" t="s" s="2">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
@@ -12754,13 +12690,13 @@
         <v>80</v>
       </c>
       <c r="K92" t="s" s="2">
-        <v>228</v>
+        <v>102</v>
       </c>
       <c r="L92" t="s" s="2">
-        <v>527</v>
+        <v>103</v>
       </c>
       <c r="M92" t="s" s="2">
-        <v>528</v>
+        <v>104</v>
       </c>
       <c r="N92" s="2"/>
       <c r="O92" s="2"/>
@@ -12787,13 +12723,13 @@
         <v>80</v>
       </c>
       <c r="X92" t="s" s="2">
-        <v>172</v>
+        <v>80</v>
       </c>
       <c r="Y92" t="s" s="2">
-        <v>529</v>
+        <v>80</v>
       </c>
       <c r="Z92" t="s" s="2">
-        <v>530</v>
+        <v>80</v>
       </c>
       <c r="AA92" t="s" s="2">
         <v>80</v>
@@ -12811,7 +12747,7 @@
         <v>80</v>
       </c>
       <c r="AF92" t="s" s="2">
-        <v>526</v>
+        <v>105</v>
       </c>
       <c r="AG92" t="s" s="2">
         <v>78</v>
@@ -12823,7 +12759,7 @@
         <v>80</v>
       </c>
       <c r="AJ92" t="s" s="2">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AK92" t="s" s="2">
         <v>80</v>
@@ -12840,21 +12776,21 @@
     </row>
     <row r="93">
       <c r="A93" t="s" s="2">
-        <v>531</v>
+        <v>526</v>
       </c>
       <c r="B93" t="s" s="2">
-        <v>531</v>
+        <v>526</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
-        <v>80</v>
+        <v>108</v>
       </c>
       <c r="E93" s="2"/>
       <c r="F93" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G93" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H93" t="s" s="2">
         <v>80</v>
@@ -12866,15 +12802,17 @@
         <v>80</v>
       </c>
       <c r="K93" t="s" s="2">
-        <v>532</v>
+        <v>109</v>
       </c>
       <c r="L93" t="s" s="2">
-        <v>533</v>
+        <v>110</v>
       </c>
       <c r="M93" t="s" s="2">
-        <v>534</v>
-      </c>
-      <c r="N93" s="2"/>
+        <v>111</v>
+      </c>
+      <c r="N93" t="s" s="2">
+        <v>112</v>
+      </c>
       <c r="O93" s="2"/>
       <c r="P93" t="s" s="2">
         <v>80</v>
@@ -12923,25 +12861,25 @@
         <v>80</v>
       </c>
       <c r="AF93" t="s" s="2">
-        <v>531</v>
+        <v>116</v>
       </c>
       <c r="AG93" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH93" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI93" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ93" t="s" s="2">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="AK93" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL93" t="s" s="2">
-        <v>535</v>
+        <v>106</v>
       </c>
       <c r="AM93" t="s" s="2">
         <v>80</v>
@@ -12952,44 +12890,46 @@
     </row>
     <row r="94">
       <c r="A94" t="s" s="2">
-        <v>536</v>
+        <v>527</v>
       </c>
       <c r="B94" t="s" s="2">
-        <v>536</v>
+        <v>527</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
-        <v>80</v>
+        <v>286</v>
       </c>
       <c r="E94" s="2"/>
       <c r="F94" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G94" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H94" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I94" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="J94" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="K94" t="s" s="2">
-        <v>537</v>
+        <v>109</v>
       </c>
       <c r="L94" t="s" s="2">
-        <v>538</v>
+        <v>287</v>
       </c>
       <c r="M94" t="s" s="2">
-        <v>539</v>
+        <v>288</v>
       </c>
       <c r="N94" t="s" s="2">
-        <v>540</v>
-      </c>
-      <c r="O94" s="2"/>
+        <v>112</v>
+      </c>
+      <c r="O94" t="s" s="2">
+        <v>205</v>
+      </c>
       <c r="P94" t="s" s="2">
         <v>80</v>
       </c>
@@ -13037,7 +12977,7 @@
         <v>80</v>
       </c>
       <c r="AF94" t="s" s="2">
-        <v>536</v>
+        <v>289</v>
       </c>
       <c r="AG94" t="s" s="2">
         <v>78</v>
@@ -13049,13 +12989,13 @@
         <v>80</v>
       </c>
       <c r="AJ94" t="s" s="2">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="AK94" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL94" t="s" s="2">
-        <v>541</v>
+        <v>191</v>
       </c>
       <c r="AM94" t="s" s="2">
         <v>80</v>
@@ -13066,10 +13006,10 @@
     </row>
     <row r="95">
       <c r="A95" t="s" s="2">
-        <v>542</v>
+        <v>528</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>542</v>
+        <v>528</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
@@ -13092,17 +13032,15 @@
         <v>80</v>
       </c>
       <c r="K95" t="s" s="2">
-        <v>279</v>
+        <v>208</v>
       </c>
       <c r="L95" t="s" s="2">
-        <v>543</v>
+        <v>529</v>
       </c>
       <c r="M95" t="s" s="2">
-        <v>544</v>
-      </c>
-      <c r="N95" t="s" s="2">
-        <v>545</v>
-      </c>
+        <v>530</v>
+      </c>
+      <c r="N95" s="2"/>
       <c r="O95" s="2"/>
       <c r="P95" t="s" s="2">
         <v>80</v>
@@ -13151,7 +13089,7 @@
         <v>80</v>
       </c>
       <c r="AF95" t="s" s="2">
-        <v>542</v>
+        <v>528</v>
       </c>
       <c r="AG95" t="s" s="2">
         <v>78</v>
@@ -13169,21 +13107,21 @@
         <v>80</v>
       </c>
       <c r="AL95" t="s" s="2">
-        <v>546</v>
+        <v>212</v>
       </c>
       <c r="AM95" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN95" t="s" s="2">
-        <v>80</v>
+        <v>531</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="s" s="2">
-        <v>547</v>
+        <v>532</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>547</v>
+        <v>532</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -13292,10 +13230,10 @@
     </row>
     <row r="97">
       <c r="A97" t="s" s="2">
-        <v>548</v>
+        <v>533</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>548</v>
+        <v>533</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -13365,16 +13303,16 @@
         <v>80</v>
       </c>
       <c r="AB97" t="s" s="2">
-        <v>80</v>
+        <v>113</v>
       </c>
       <c r="AC97" t="s" s="2">
-        <v>80</v>
+        <v>114</v>
       </c>
       <c r="AD97" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE97" t="s" s="2">
-        <v>80</v>
+        <v>115</v>
       </c>
       <c r="AF97" t="s" s="2">
         <v>116</v>
@@ -13406,21 +13344,21 @@
     </row>
     <row r="98">
       <c r="A98" t="s" s="2">
-        <v>549</v>
+        <v>534</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>549</v>
+        <v>534</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
-        <v>286</v>
+        <v>80</v>
       </c>
       <c r="E98" s="2"/>
       <c r="F98" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G98" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H98" t="s" s="2">
         <v>80</v>
@@ -13432,19 +13370,19 @@
         <v>89</v>
       </c>
       <c r="K98" t="s" s="2">
-        <v>109</v>
+        <v>168</v>
       </c>
       <c r="L98" t="s" s="2">
-        <v>287</v>
+        <v>218</v>
       </c>
       <c r="M98" t="s" s="2">
-        <v>288</v>
+        <v>219</v>
       </c>
       <c r="N98" t="s" s="2">
-        <v>112</v>
+        <v>220</v>
       </c>
       <c r="O98" t="s" s="2">
-        <v>205</v>
+        <v>221</v>
       </c>
       <c r="P98" t="s" s="2">
         <v>80</v>
@@ -13469,13 +13407,13 @@
         <v>80</v>
       </c>
       <c r="X98" t="s" s="2">
-        <v>80</v>
+        <v>222</v>
       </c>
       <c r="Y98" t="s" s="2">
-        <v>80</v>
+        <v>223</v>
       </c>
       <c r="Z98" t="s" s="2">
-        <v>80</v>
+        <v>224</v>
       </c>
       <c r="AA98" t="s" s="2">
         <v>80</v>
@@ -13493,39 +13431,39 @@
         <v>80</v>
       </c>
       <c r="AF98" t="s" s="2">
-        <v>289</v>
+        <v>225</v>
       </c>
       <c r="AG98" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH98" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI98" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ98" t="s" s="2">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="AK98" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL98" t="s" s="2">
+        <v>226</v>
+      </c>
+      <c r="AM98" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN98" t="s" s="2">
         <v>191</v>
-      </c>
-      <c r="AM98" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN98" t="s" s="2">
-        <v>80</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="s" s="2">
-        <v>550</v>
+        <v>535</v>
       </c>
       <c r="B99" t="s" s="2">
-        <v>550</v>
+        <v>535</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" t="s" s="2">
@@ -13533,7 +13471,7 @@
       </c>
       <c r="E99" s="2"/>
       <c r="F99" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G99" t="s" s="2">
         <v>88</v>
@@ -13545,19 +13483,23 @@
         <v>80</v>
       </c>
       <c r="J99" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="K99" t="s" s="2">
-        <v>208</v>
+        <v>228</v>
       </c>
       <c r="L99" t="s" s="2">
-        <v>551</v>
+        <v>229</v>
       </c>
       <c r="M99" t="s" s="2">
-        <v>552</v>
-      </c>
-      <c r="N99" s="2"/>
-      <c r="O99" s="2"/>
+        <v>536</v>
+      </c>
+      <c r="N99" t="s" s="2">
+        <v>231</v>
+      </c>
+      <c r="O99" t="s" s="2">
+        <v>232</v>
+      </c>
       <c r="P99" t="s" s="2">
         <v>80</v>
       </c>
@@ -13581,13 +13523,11 @@
         <v>80</v>
       </c>
       <c r="X99" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y99" t="s" s="2">
-        <v>80</v>
-      </c>
+        <v>150</v>
+      </c>
+      <c r="Y99" s="2"/>
       <c r="Z99" t="s" s="2">
-        <v>80</v>
+        <v>233</v>
       </c>
       <c r="AA99" t="s" s="2">
         <v>80</v>
@@ -13605,7 +13545,7 @@
         <v>80</v>
       </c>
       <c r="AF99" t="s" s="2">
-        <v>550</v>
+        <v>234</v>
       </c>
       <c r="AG99" t="s" s="2">
         <v>78</v>
@@ -13623,21 +13563,21 @@
         <v>80</v>
       </c>
       <c r="AL99" t="s" s="2">
-        <v>212</v>
+        <v>226</v>
       </c>
       <c r="AM99" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN99" t="s" s="2">
-        <v>553</v>
+        <v>235</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="s" s="2">
-        <v>554</v>
+        <v>537</v>
       </c>
       <c r="B100" t="s" s="2">
-        <v>554</v>
+        <v>537</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -13645,7 +13585,7 @@
       </c>
       <c r="E100" s="2"/>
       <c r="F100" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G100" t="s" s="2">
         <v>88</v>
@@ -13657,31 +13597,35 @@
         <v>80</v>
       </c>
       <c r="J100" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="K100" t="s" s="2">
-        <v>102</v>
+        <v>130</v>
       </c>
       <c r="L100" t="s" s="2">
-        <v>103</v>
+        <v>237</v>
       </c>
       <c r="M100" t="s" s="2">
-        <v>104</v>
-      </c>
-      <c r="N100" s="2"/>
-      <c r="O100" s="2"/>
+        <v>538</v>
+      </c>
+      <c r="N100" t="s" s="2">
+        <v>239</v>
+      </c>
+      <c r="O100" t="s" s="2">
+        <v>240</v>
+      </c>
       <c r="P100" t="s" s="2">
         <v>80</v>
       </c>
       <c r="Q100" s="2"/>
       <c r="R100" t="s" s="2">
-        <v>80</v>
+        <v>539</v>
       </c>
       <c r="S100" t="s" s="2">
         <v>80</v>
       </c>
       <c r="T100" t="s" s="2">
-        <v>80</v>
+        <v>241</v>
       </c>
       <c r="U100" t="s" s="2">
         <v>80</v>
@@ -13717,7 +13661,7 @@
         <v>80</v>
       </c>
       <c r="AF100" t="s" s="2">
-        <v>105</v>
+        <v>242</v>
       </c>
       <c r="AG100" t="s" s="2">
         <v>78</v>
@@ -13729,38 +13673,38 @@
         <v>80</v>
       </c>
       <c r="AJ100" t="s" s="2">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="AK100" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL100" t="s" s="2">
-        <v>106</v>
+        <v>243</v>
       </c>
       <c r="AM100" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN100" t="s" s="2">
-        <v>80</v>
+        <v>244</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="s" s="2">
-        <v>555</v>
+        <v>540</v>
       </c>
       <c r="B101" t="s" s="2">
-        <v>555</v>
+        <v>540</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" t="s" s="2">
-        <v>108</v>
+        <v>80</v>
       </c>
       <c r="E101" s="2"/>
       <c r="F101" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G101" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H101" t="s" s="2">
         <v>80</v>
@@ -13769,19 +13713,19 @@
         <v>80</v>
       </c>
       <c r="J101" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="K101" t="s" s="2">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="L101" t="s" s="2">
-        <v>110</v>
+        <v>246</v>
       </c>
       <c r="M101" t="s" s="2">
-        <v>111</v>
+        <v>247</v>
       </c>
       <c r="N101" t="s" s="2">
-        <v>112</v>
+        <v>248</v>
       </c>
       <c r="O101" s="2"/>
       <c r="P101" t="s" s="2">
@@ -13795,7 +13739,7 @@
         <v>80</v>
       </c>
       <c r="T101" t="s" s="2">
-        <v>80</v>
+        <v>249</v>
       </c>
       <c r="U101" t="s" s="2">
         <v>80</v>
@@ -13819,51 +13763,51 @@
         <v>80</v>
       </c>
       <c r="AB101" t="s" s="2">
-        <v>113</v>
+        <v>80</v>
       </c>
       <c r="AC101" t="s" s="2">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="AD101" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE101" t="s" s="2">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="AF101" t="s" s="2">
-        <v>116</v>
+        <v>250</v>
       </c>
       <c r="AG101" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH101" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI101" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ101" t="s" s="2">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="AK101" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL101" t="s" s="2">
-        <v>106</v>
+        <v>251</v>
       </c>
       <c r="AM101" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN101" t="s" s="2">
-        <v>80</v>
+        <v>252</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="s" s="2">
-        <v>556</v>
+        <v>541</v>
       </c>
       <c r="B102" t="s" s="2">
-        <v>556</v>
+        <v>541</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" t="s" s="2">
@@ -13880,26 +13824,22 @@
         <v>80</v>
       </c>
       <c r="I102" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="J102" t="s" s="2">
         <v>89</v>
       </c>
       <c r="K102" t="s" s="2">
-        <v>168</v>
+        <v>254</v>
       </c>
       <c r="L102" t="s" s="2">
-        <v>218</v>
+        <v>255</v>
       </c>
       <c r="M102" t="s" s="2">
-        <v>219</v>
-      </c>
-      <c r="N102" t="s" s="2">
-        <v>220</v>
-      </c>
-      <c r="O102" t="s" s="2">
-        <v>221</v>
-      </c>
+        <v>256</v>
+      </c>
+      <c r="N102" s="2"/>
+      <c r="O102" s="2"/>
       <c r="P102" t="s" s="2">
         <v>80</v>
       </c>
@@ -13923,13 +13863,13 @@
         <v>80</v>
       </c>
       <c r="X102" t="s" s="2">
-        <v>222</v>
+        <v>80</v>
       </c>
       <c r="Y102" t="s" s="2">
-        <v>223</v>
+        <v>80</v>
       </c>
       <c r="Z102" t="s" s="2">
-        <v>224</v>
+        <v>80</v>
       </c>
       <c r="AA102" t="s" s="2">
         <v>80</v>
@@ -13947,7 +13887,7 @@
         <v>80</v>
       </c>
       <c r="AF102" t="s" s="2">
-        <v>225</v>
+        <v>257</v>
       </c>
       <c r="AG102" t="s" s="2">
         <v>78</v>
@@ -13965,21 +13905,21 @@
         <v>80</v>
       </c>
       <c r="AL102" t="s" s="2">
-        <v>226</v>
+        <v>258</v>
       </c>
       <c r="AM102" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN102" t="s" s="2">
-        <v>191</v>
+        <v>259</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="s" s="2">
-        <v>557</v>
+        <v>542</v>
       </c>
       <c r="B103" t="s" s="2">
-        <v>557</v>
+        <v>542</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" t="s" s="2">
@@ -13987,7 +13927,7 @@
       </c>
       <c r="E103" s="2"/>
       <c r="F103" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="G103" t="s" s="2">
         <v>88</v>
@@ -14002,20 +13942,18 @@
         <v>89</v>
       </c>
       <c r="K103" t="s" s="2">
-        <v>228</v>
+        <v>261</v>
       </c>
       <c r="L103" t="s" s="2">
-        <v>229</v>
+        <v>262</v>
       </c>
       <c r="M103" t="s" s="2">
-        <v>558</v>
+        <v>263</v>
       </c>
       <c r="N103" t="s" s="2">
-        <v>231</v>
-      </c>
-      <c r="O103" t="s" s="2">
-        <v>232</v>
-      </c>
+        <v>264</v>
+      </c>
+      <c r="O103" s="2"/>
       <c r="P103" t="s" s="2">
         <v>80</v>
       </c>
@@ -14039,11 +13977,13 @@
         <v>80</v>
       </c>
       <c r="X103" t="s" s="2">
-        <v>150</v>
-      </c>
-      <c r="Y103" s="2"/>
+        <v>80</v>
+      </c>
+      <c r="Y103" t="s" s="2">
+        <v>80</v>
+      </c>
       <c r="Z103" t="s" s="2">
-        <v>233</v>
+        <v>80</v>
       </c>
       <c r="AA103" t="s" s="2">
         <v>80</v>
@@ -14061,7 +14001,7 @@
         <v>80</v>
       </c>
       <c r="AF103" t="s" s="2">
-        <v>234</v>
+        <v>265</v>
       </c>
       <c r="AG103" t="s" s="2">
         <v>78</v>
@@ -14079,21 +14019,21 @@
         <v>80</v>
       </c>
       <c r="AL103" t="s" s="2">
-        <v>226</v>
+        <v>266</v>
       </c>
       <c r="AM103" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN103" t="s" s="2">
-        <v>235</v>
+        <v>267</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="s" s="2">
-        <v>559</v>
+        <v>543</v>
       </c>
       <c r="B104" t="s" s="2">
-        <v>559</v>
+        <v>543</v>
       </c>
       <c r="C104" s="2"/>
       <c r="D104" t="s" s="2">
@@ -14101,7 +14041,7 @@
       </c>
       <c r="E104" s="2"/>
       <c r="F104" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="G104" t="s" s="2">
         <v>88</v>
@@ -14113,35 +14053,31 @@
         <v>80</v>
       </c>
       <c r="J104" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="K104" t="s" s="2">
-        <v>130</v>
+        <v>544</v>
       </c>
       <c r="L104" t="s" s="2">
-        <v>237</v>
+        <v>545</v>
       </c>
       <c r="M104" t="s" s="2">
-        <v>560</v>
-      </c>
-      <c r="N104" t="s" s="2">
-        <v>239</v>
-      </c>
-      <c r="O104" t="s" s="2">
-        <v>240</v>
-      </c>
+        <v>546</v>
+      </c>
+      <c r="N104" s="2"/>
+      <c r="O104" s="2"/>
       <c r="P104" t="s" s="2">
         <v>80</v>
       </c>
       <c r="Q104" s="2"/>
       <c r="R104" t="s" s="2">
-        <v>561</v>
+        <v>80</v>
       </c>
       <c r="S104" t="s" s="2">
         <v>80</v>
       </c>
       <c r="T104" t="s" s="2">
-        <v>241</v>
+        <v>80</v>
       </c>
       <c r="U104" t="s" s="2">
         <v>80</v>
@@ -14177,7 +14113,7 @@
         <v>80</v>
       </c>
       <c r="AF104" t="s" s="2">
-        <v>242</v>
+        <v>543</v>
       </c>
       <c r="AG104" t="s" s="2">
         <v>78</v>
@@ -14195,21 +14131,21 @@
         <v>80</v>
       </c>
       <c r="AL104" t="s" s="2">
-        <v>243</v>
+        <v>547</v>
       </c>
       <c r="AM104" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN104" t="s" s="2">
-        <v>244</v>
+        <v>80</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="s" s="2">
-        <v>562</v>
+        <v>548</v>
       </c>
       <c r="B105" t="s" s="2">
-        <v>562</v>
+        <v>548</v>
       </c>
       <c r="C105" s="2"/>
       <c r="D105" t="s" s="2">
@@ -14217,7 +14153,7 @@
       </c>
       <c r="E105" s="2"/>
       <c r="F105" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="G105" t="s" s="2">
         <v>88</v>
@@ -14229,20 +14165,18 @@
         <v>80</v>
       </c>
       <c r="J105" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="K105" t="s" s="2">
-        <v>102</v>
+        <v>228</v>
       </c>
       <c r="L105" t="s" s="2">
-        <v>246</v>
+        <v>549</v>
       </c>
       <c r="M105" t="s" s="2">
-        <v>247</v>
-      </c>
-      <c r="N105" t="s" s="2">
-        <v>248</v>
-      </c>
+        <v>550</v>
+      </c>
+      <c r="N105" s="2"/>
       <c r="O105" s="2"/>
       <c r="P105" t="s" s="2">
         <v>80</v>
@@ -14255,7 +14189,7 @@
         <v>80</v>
       </c>
       <c r="T105" t="s" s="2">
-        <v>249</v>
+        <v>80</v>
       </c>
       <c r="U105" t="s" s="2">
         <v>80</v>
@@ -14267,13 +14201,13 @@
         <v>80</v>
       </c>
       <c r="X105" t="s" s="2">
-        <v>80</v>
+        <v>172</v>
       </c>
       <c r="Y105" t="s" s="2">
-        <v>80</v>
+        <v>551</v>
       </c>
       <c r="Z105" t="s" s="2">
-        <v>80</v>
+        <v>552</v>
       </c>
       <c r="AA105" t="s" s="2">
         <v>80</v>
@@ -14291,7 +14225,7 @@
         <v>80</v>
       </c>
       <c r="AF105" t="s" s="2">
-        <v>250</v>
+        <v>548</v>
       </c>
       <c r="AG105" t="s" s="2">
         <v>78</v>
@@ -14309,21 +14243,21 @@
         <v>80</v>
       </c>
       <c r="AL105" t="s" s="2">
-        <v>251</v>
+        <v>553</v>
       </c>
       <c r="AM105" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN105" t="s" s="2">
-        <v>252</v>
+        <v>554</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="s" s="2">
-        <v>563</v>
+        <v>555</v>
       </c>
       <c r="B106" t="s" s="2">
-        <v>563</v>
+        <v>555</v>
       </c>
       <c r="C106" s="2"/>
       <c r="D106" t="s" s="2">
@@ -14343,16 +14277,16 @@
         <v>80</v>
       </c>
       <c r="J106" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="K106" t="s" s="2">
-        <v>254</v>
+        <v>228</v>
       </c>
       <c r="L106" t="s" s="2">
-        <v>255</v>
+        <v>556</v>
       </c>
       <c r="M106" t="s" s="2">
-        <v>256</v>
+        <v>557</v>
       </c>
       <c r="N106" s="2"/>
       <c r="O106" s="2"/>
@@ -14379,13 +14313,13 @@
         <v>80</v>
       </c>
       <c r="X106" t="s" s="2">
-        <v>80</v>
+        <v>158</v>
       </c>
       <c r="Y106" t="s" s="2">
-        <v>80</v>
+        <v>558</v>
       </c>
       <c r="Z106" t="s" s="2">
-        <v>80</v>
+        <v>559</v>
       </c>
       <c r="AA106" t="s" s="2">
         <v>80</v>
@@ -14403,7 +14337,7 @@
         <v>80</v>
       </c>
       <c r="AF106" t="s" s="2">
-        <v>257</v>
+        <v>555</v>
       </c>
       <c r="AG106" t="s" s="2">
         <v>78</v>
@@ -14421,21 +14355,21 @@
         <v>80</v>
       </c>
       <c r="AL106" t="s" s="2">
-        <v>258</v>
+        <v>106</v>
       </c>
       <c r="AM106" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN106" t="s" s="2">
-        <v>259</v>
+        <v>560</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="s" s="2">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="B107" t="s" s="2">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="C107" s="2"/>
       <c r="D107" t="s" s="2">
@@ -14446,7 +14380,7 @@
         <v>78</v>
       </c>
       <c r="G107" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H107" t="s" s="2">
         <v>80</v>
@@ -14455,21 +14389,23 @@
         <v>80</v>
       </c>
       <c r="J107" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="K107" t="s" s="2">
-        <v>261</v>
+        <v>228</v>
       </c>
       <c r="L107" t="s" s="2">
-        <v>262</v>
+        <v>562</v>
       </c>
       <c r="M107" t="s" s="2">
-        <v>263</v>
+        <v>563</v>
       </c>
       <c r="N107" t="s" s="2">
-        <v>264</v>
-      </c>
-      <c r="O107" s="2"/>
+        <v>564</v>
+      </c>
+      <c r="O107" t="s" s="2">
+        <v>565</v>
+      </c>
       <c r="P107" t="s" s="2">
         <v>80</v>
       </c>
@@ -14493,13 +14429,13 @@
         <v>80</v>
       </c>
       <c r="X107" t="s" s="2">
-        <v>80</v>
+        <v>158</v>
       </c>
       <c r="Y107" t="s" s="2">
-        <v>80</v>
+        <v>566</v>
       </c>
       <c r="Z107" t="s" s="2">
-        <v>80</v>
+        <v>567</v>
       </c>
       <c r="AA107" t="s" s="2">
         <v>80</v>
@@ -14517,13 +14453,13 @@
         <v>80</v>
       </c>
       <c r="AF107" t="s" s="2">
-        <v>265</v>
+        <v>561</v>
       </c>
       <c r="AG107" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH107" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI107" t="s" s="2">
         <v>80</v>
@@ -14535,21 +14471,21 @@
         <v>80</v>
       </c>
       <c r="AL107" t="s" s="2">
-        <v>266</v>
+        <v>568</v>
       </c>
       <c r="AM107" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN107" t="s" s="2">
-        <v>267</v>
+        <v>569</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="s" s="2">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="B108" t="s" s="2">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="C108" s="2"/>
       <c r="D108" t="s" s="2">
@@ -14560,7 +14496,7 @@
         <v>78</v>
       </c>
       <c r="G108" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H108" t="s" s="2">
         <v>80</v>
@@ -14572,13 +14508,13 @@
         <v>80</v>
       </c>
       <c r="K108" t="s" s="2">
-        <v>566</v>
+        <v>228</v>
       </c>
       <c r="L108" t="s" s="2">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="M108" t="s" s="2">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="N108" s="2"/>
       <c r="O108" s="2"/>
@@ -14605,13 +14541,13 @@
         <v>80</v>
       </c>
       <c r="X108" t="s" s="2">
-        <v>80</v>
+        <v>172</v>
       </c>
       <c r="Y108" t="s" s="2">
-        <v>80</v>
+        <v>573</v>
       </c>
       <c r="Z108" t="s" s="2">
-        <v>80</v>
+        <v>574</v>
       </c>
       <c r="AA108" t="s" s="2">
         <v>80</v>
@@ -14629,13 +14565,13 @@
         <v>80</v>
       </c>
       <c r="AF108" t="s" s="2">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="AG108" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH108" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI108" t="s" s="2">
         <v>80</v>
@@ -14647,21 +14583,21 @@
         <v>80</v>
       </c>
       <c r="AL108" t="s" s="2">
-        <v>569</v>
+        <v>575</v>
       </c>
       <c r="AM108" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN108" t="s" s="2">
-        <v>80</v>
+        <v>576</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="s" s="2">
-        <v>570</v>
+        <v>577</v>
       </c>
       <c r="B109" t="s" s="2">
-        <v>570</v>
+        <v>577</v>
       </c>
       <c r="C109" s="2"/>
       <c r="D109" t="s" s="2">
@@ -14672,7 +14608,7 @@
         <v>78</v>
       </c>
       <c r="G109" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H109" t="s" s="2">
         <v>80</v>
@@ -14687,10 +14623,10 @@
         <v>228</v>
       </c>
       <c r="L109" t="s" s="2">
-        <v>571</v>
+        <v>578</v>
       </c>
       <c r="M109" t="s" s="2">
-        <v>572</v>
+        <v>579</v>
       </c>
       <c r="N109" s="2"/>
       <c r="O109" s="2"/>
@@ -14720,10 +14656,10 @@
         <v>172</v>
       </c>
       <c r="Y109" t="s" s="2">
-        <v>573</v>
+        <v>580</v>
       </c>
       <c r="Z109" t="s" s="2">
-        <v>574</v>
+        <v>581</v>
       </c>
       <c r="AA109" t="s" s="2">
         <v>80</v>
@@ -14741,13 +14677,13 @@
         <v>80</v>
       </c>
       <c r="AF109" t="s" s="2">
-        <v>570</v>
+        <v>577</v>
       </c>
       <c r="AG109" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH109" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI109" t="s" s="2">
         <v>80</v>
@@ -14759,21 +14695,21 @@
         <v>80</v>
       </c>
       <c r="AL109" t="s" s="2">
-        <v>575</v>
+        <v>582</v>
       </c>
       <c r="AM109" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN109" t="s" s="2">
-        <v>576</v>
+        <v>583</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="s" s="2">
-        <v>577</v>
+        <v>584</v>
       </c>
       <c r="B110" t="s" s="2">
-        <v>577</v>
+        <v>584</v>
       </c>
       <c r="C110" s="2"/>
       <c r="D110" t="s" s="2">
@@ -14796,13 +14732,13 @@
         <v>80</v>
       </c>
       <c r="K110" t="s" s="2">
-        <v>228</v>
+        <v>544</v>
       </c>
       <c r="L110" t="s" s="2">
-        <v>578</v>
+        <v>585</v>
       </c>
       <c r="M110" t="s" s="2">
-        <v>579</v>
+        <v>586</v>
       </c>
       <c r="N110" s="2"/>
       <c r="O110" s="2"/>
@@ -14829,13 +14765,13 @@
         <v>80</v>
       </c>
       <c r="X110" t="s" s="2">
-        <v>158</v>
+        <v>80</v>
       </c>
       <c r="Y110" t="s" s="2">
-        <v>580</v>
+        <v>80</v>
       </c>
       <c r="Z110" t="s" s="2">
-        <v>581</v>
+        <v>80</v>
       </c>
       <c r="AA110" t="s" s="2">
         <v>80</v>
@@ -14853,7 +14789,7 @@
         <v>80</v>
       </c>
       <c r="AF110" t="s" s="2">
-        <v>577</v>
+        <v>584</v>
       </c>
       <c r="AG110" t="s" s="2">
         <v>78</v>
@@ -14871,21 +14807,21 @@
         <v>80</v>
       </c>
       <c r="AL110" t="s" s="2">
-        <v>106</v>
+        <v>587</v>
       </c>
       <c r="AM110" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN110" t="s" s="2">
-        <v>582</v>
+        <v>588</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="s" s="2">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="B111" t="s" s="2">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="C111" s="2"/>
       <c r="D111" t="s" s="2">
@@ -14896,7 +14832,7 @@
         <v>78</v>
       </c>
       <c r="G111" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H111" t="s" s="2">
         <v>80</v>
@@ -14911,17 +14847,13 @@
         <v>228</v>
       </c>
       <c r="L111" t="s" s="2">
-        <v>584</v>
+        <v>590</v>
       </c>
       <c r="M111" t="s" s="2">
-        <v>585</v>
-      </c>
-      <c r="N111" t="s" s="2">
-        <v>586</v>
-      </c>
-      <c r="O111" t="s" s="2">
-        <v>587</v>
-      </c>
+        <v>591</v>
+      </c>
+      <c r="N111" s="2"/>
+      <c r="O111" s="2"/>
       <c r="P111" t="s" s="2">
         <v>80</v>
       </c>
@@ -14947,35 +14879,33 @@
       <c r="X111" t="s" s="2">
         <v>158</v>
       </c>
-      <c r="Y111" t="s" s="2">
-        <v>588</v>
-      </c>
+      <c r="Y111" s="2"/>
       <c r="Z111" t="s" s="2">
+        <v>592</v>
+      </c>
+      <c r="AA111" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB111" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC111" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD111" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE111" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF111" t="s" s="2">
         <v>589</v>
       </c>
-      <c r="AA111" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB111" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC111" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD111" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE111" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF111" t="s" s="2">
-        <v>583</v>
-      </c>
       <c r="AG111" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH111" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI111" t="s" s="2">
         <v>80</v>
@@ -14987,21 +14917,21 @@
         <v>80</v>
       </c>
       <c r="AL111" t="s" s="2">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="AM111" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN111" t="s" s="2">
-        <v>591</v>
+        <v>594</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="s" s="2">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="B112" t="s" s="2">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="C112" s="2"/>
       <c r="D112" t="s" s="2">
@@ -15009,10 +14939,10 @@
       </c>
       <c r="E112" s="2"/>
       <c r="F112" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G112" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H112" t="s" s="2">
         <v>80</v>
@@ -15024,15 +14954,17 @@
         <v>80</v>
       </c>
       <c r="K112" t="s" s="2">
-        <v>228</v>
+        <v>279</v>
       </c>
       <c r="L112" t="s" s="2">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="M112" t="s" s="2">
-        <v>594</v>
-      </c>
-      <c r="N112" s="2"/>
+        <v>597</v>
+      </c>
+      <c r="N112" t="s" s="2">
+        <v>598</v>
+      </c>
       <c r="O112" s="2"/>
       <c r="P112" t="s" s="2">
         <v>80</v>
@@ -15057,31 +14989,31 @@
         <v>80</v>
       </c>
       <c r="X112" t="s" s="2">
-        <v>172</v>
+        <v>80</v>
       </c>
       <c r="Y112" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z112" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA112" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB112" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC112" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD112" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE112" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF112" t="s" s="2">
         <v>595</v>
-      </c>
-      <c r="Z112" t="s" s="2">
-        <v>596</v>
-      </c>
-      <c r="AA112" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB112" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC112" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD112" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE112" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF112" t="s" s="2">
-        <v>592</v>
       </c>
       <c r="AG112" t="s" s="2">
         <v>78</v>
@@ -15099,21 +15031,21 @@
         <v>80</v>
       </c>
       <c r="AL112" t="s" s="2">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="AM112" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN112" t="s" s="2">
-        <v>598</v>
+        <v>80</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="s" s="2">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="B113" t="s" s="2">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="C113" s="2"/>
       <c r="D113" t="s" s="2">
@@ -15124,7 +15056,7 @@
         <v>78</v>
       </c>
       <c r="G113" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H113" t="s" s="2">
         <v>80</v>
@@ -15136,13 +15068,13 @@
         <v>80</v>
       </c>
       <c r="K113" t="s" s="2">
-        <v>228</v>
+        <v>102</v>
       </c>
       <c r="L113" t="s" s="2">
-        <v>600</v>
+        <v>103</v>
       </c>
       <c r="M113" t="s" s="2">
-        <v>601</v>
+        <v>104</v>
       </c>
       <c r="N113" s="2"/>
       <c r="O113" s="2"/>
@@ -15169,13 +15101,13 @@
         <v>80</v>
       </c>
       <c r="X113" t="s" s="2">
-        <v>172</v>
+        <v>80</v>
       </c>
       <c r="Y113" t="s" s="2">
-        <v>602</v>
+        <v>80</v>
       </c>
       <c r="Z113" t="s" s="2">
-        <v>603</v>
+        <v>80</v>
       </c>
       <c r="AA113" t="s" s="2">
         <v>80</v>
@@ -15193,50 +15125,50 @@
         <v>80</v>
       </c>
       <c r="AF113" t="s" s="2">
-        <v>599</v>
+        <v>105</v>
       </c>
       <c r="AG113" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH113" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI113" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ113" t="s" s="2">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AK113" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL113" t="s" s="2">
-        <v>604</v>
+        <v>106</v>
       </c>
       <c r="AM113" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN113" t="s" s="2">
-        <v>605</v>
+        <v>80</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="s" s="2">
-        <v>606</v>
+        <v>601</v>
       </c>
       <c r="B114" t="s" s="2">
-        <v>606</v>
+        <v>601</v>
       </c>
       <c r="C114" s="2"/>
       <c r="D114" t="s" s="2">
-        <v>80</v>
+        <v>108</v>
       </c>
       <c r="E114" s="2"/>
       <c r="F114" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G114" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H114" t="s" s="2">
         <v>80</v>
@@ -15248,15 +15180,17 @@
         <v>80</v>
       </c>
       <c r="K114" t="s" s="2">
-        <v>566</v>
+        <v>109</v>
       </c>
       <c r="L114" t="s" s="2">
-        <v>607</v>
+        <v>110</v>
       </c>
       <c r="M114" t="s" s="2">
-        <v>608</v>
-      </c>
-      <c r="N114" s="2"/>
+        <v>111</v>
+      </c>
+      <c r="N114" t="s" s="2">
+        <v>112</v>
+      </c>
       <c r="O114" s="2"/>
       <c r="P114" t="s" s="2">
         <v>80</v>
@@ -15305,71 +15239,75 @@
         <v>80</v>
       </c>
       <c r="AF114" t="s" s="2">
-        <v>606</v>
+        <v>116</v>
       </c>
       <c r="AG114" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH114" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI114" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ114" t="s" s="2">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="AK114" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL114" t="s" s="2">
-        <v>609</v>
+        <v>106</v>
       </c>
       <c r="AM114" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN114" t="s" s="2">
-        <v>610</v>
+        <v>80</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="s" s="2">
-        <v>611</v>
+        <v>602</v>
       </c>
       <c r="B115" t="s" s="2">
-        <v>611</v>
+        <v>602</v>
       </c>
       <c r="C115" s="2"/>
       <c r="D115" t="s" s="2">
-        <v>80</v>
+        <v>286</v>
       </c>
       <c r="E115" s="2"/>
       <c r="F115" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G115" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="H115" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I115" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="J115" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="K115" t="s" s="2">
-        <v>228</v>
+        <v>109</v>
       </c>
       <c r="L115" t="s" s="2">
-        <v>612</v>
+        <v>287</v>
       </c>
       <c r="M115" t="s" s="2">
-        <v>613</v>
-      </c>
-      <c r="N115" s="2"/>
-      <c r="O115" s="2"/>
+        <v>288</v>
+      </c>
+      <c r="N115" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="O115" t="s" s="2">
+        <v>205</v>
+      </c>
       <c r="P115" t="s" s="2">
         <v>80</v>
       </c>
@@ -15393,11 +15331,13 @@
         <v>80</v>
       </c>
       <c r="X115" t="s" s="2">
-        <v>158</v>
-      </c>
-      <c r="Y115" s="2"/>
+        <v>80</v>
+      </c>
+      <c r="Y115" t="s" s="2">
+        <v>80</v>
+      </c>
       <c r="Z115" t="s" s="2">
-        <v>614</v>
+        <v>80</v>
       </c>
       <c r="AA115" t="s" s="2">
         <v>80</v>
@@ -15415,39 +15355,39 @@
         <v>80</v>
       </c>
       <c r="AF115" t="s" s="2">
-        <v>611</v>
+        <v>289</v>
       </c>
       <c r="AG115" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH115" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AI115" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ115" t="s" s="2">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="AK115" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL115" t="s" s="2">
-        <v>615</v>
+        <v>191</v>
       </c>
       <c r="AM115" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN115" t="s" s="2">
-        <v>616</v>
+        <v>80</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="s" s="2">
-        <v>617</v>
+        <v>603</v>
       </c>
       <c r="B116" t="s" s="2">
-        <v>617</v>
+        <v>603</v>
       </c>
       <c r="C116" s="2"/>
       <c r="D116" t="s" s="2">
@@ -15470,17 +15410,15 @@
         <v>80</v>
       </c>
       <c r="K116" t="s" s="2">
-        <v>279</v>
+        <v>604</v>
       </c>
       <c r="L116" t="s" s="2">
-        <v>618</v>
+        <v>605</v>
       </c>
       <c r="M116" t="s" s="2">
-        <v>619</v>
-      </c>
-      <c r="N116" t="s" s="2">
-        <v>620</v>
-      </c>
+        <v>606</v>
+      </c>
+      <c r="N116" s="2"/>
       <c r="O116" s="2"/>
       <c r="P116" t="s" s="2">
         <v>80</v>
@@ -15529,13 +15467,13 @@
         <v>80</v>
       </c>
       <c r="AF116" t="s" s="2">
-        <v>617</v>
+        <v>603</v>
       </c>
       <c r="AG116" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="AH116" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI116" t="s" s="2">
         <v>80</v>
@@ -15544,24 +15482,24 @@
         <v>100</v>
       </c>
       <c r="AK116" t="s" s="2">
-        <v>80</v>
+        <v>607</v>
       </c>
       <c r="AL116" t="s" s="2">
-        <v>621</v>
+        <v>427</v>
       </c>
       <c r="AM116" t="s" s="2">
-        <v>80</v>
+        <v>608</v>
       </c>
       <c r="AN116" t="s" s="2">
-        <v>80</v>
+        <v>609</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="s" s="2">
-        <v>622</v>
+        <v>610</v>
       </c>
       <c r="B117" t="s" s="2">
-        <v>622</v>
+        <v>610</v>
       </c>
       <c r="C117" s="2"/>
       <c r="D117" t="s" s="2">
@@ -15584,15 +15522,17 @@
         <v>80</v>
       </c>
       <c r="K117" t="s" s="2">
-        <v>102</v>
+        <v>168</v>
       </c>
       <c r="L117" t="s" s="2">
-        <v>103</v>
+        <v>611</v>
       </c>
       <c r="M117" t="s" s="2">
-        <v>104</v>
-      </c>
-      <c r="N117" s="2"/>
+        <v>612</v>
+      </c>
+      <c r="N117" t="s" s="2">
+        <v>613</v>
+      </c>
       <c r="O117" s="2"/>
       <c r="P117" t="s" s="2">
         <v>80</v>
@@ -15617,13 +15557,13 @@
         <v>80</v>
       </c>
       <c r="X117" t="s" s="2">
-        <v>80</v>
+        <v>222</v>
       </c>
       <c r="Y117" t="s" s="2">
-        <v>80</v>
+        <v>614</v>
       </c>
       <c r="Z117" t="s" s="2">
-        <v>80</v>
+        <v>615</v>
       </c>
       <c r="AA117" t="s" s="2">
         <v>80</v>
@@ -15641,7 +15581,7 @@
         <v>80</v>
       </c>
       <c r="AF117" t="s" s="2">
-        <v>105</v>
+        <v>610</v>
       </c>
       <c r="AG117" t="s" s="2">
         <v>78</v>
@@ -15653,13 +15593,13 @@
         <v>80</v>
       </c>
       <c r="AJ117" t="s" s="2">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="AK117" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL117" t="s" s="2">
-        <v>106</v>
+        <v>616</v>
       </c>
       <c r="AM117" t="s" s="2">
         <v>80</v>
@@ -15670,21 +15610,21 @@
     </row>
     <row r="118">
       <c r="A118" t="s" s="2">
-        <v>623</v>
+        <v>617</v>
       </c>
       <c r="B118" t="s" s="2">
-        <v>623</v>
+        <v>617</v>
       </c>
       <c r="C118" s="2"/>
       <c r="D118" t="s" s="2">
-        <v>108</v>
+        <v>80</v>
       </c>
       <c r="E118" s="2"/>
       <c r="F118" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G118" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H118" t="s" s="2">
         <v>80</v>
@@ -15696,16 +15636,16 @@
         <v>80</v>
       </c>
       <c r="K118" t="s" s="2">
-        <v>109</v>
+        <v>228</v>
       </c>
       <c r="L118" t="s" s="2">
-        <v>110</v>
+        <v>618</v>
       </c>
       <c r="M118" t="s" s="2">
-        <v>111</v>
+        <v>619</v>
       </c>
       <c r="N118" t="s" s="2">
-        <v>112</v>
+        <v>620</v>
       </c>
       <c r="O118" s="2"/>
       <c r="P118" t="s" s="2">
@@ -15731,13 +15671,11 @@
         <v>80</v>
       </c>
       <c r="X118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y118" t="s" s="2">
-        <v>80</v>
-      </c>
+        <v>158</v>
+      </c>
+      <c r="Y118" s="2"/>
       <c r="Z118" t="s" s="2">
-        <v>80</v>
+        <v>621</v>
       </c>
       <c r="AA118" t="s" s="2">
         <v>80</v>
@@ -15755,25 +15693,25 @@
         <v>80</v>
       </c>
       <c r="AF118" t="s" s="2">
-        <v>116</v>
+        <v>617</v>
       </c>
       <c r="AG118" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH118" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI118" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ118" t="s" s="2">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="AK118" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL118" t="s" s="2">
-        <v>106</v>
+        <v>80</v>
       </c>
       <c r="AM118" t="s" s="2">
         <v>80</v>
@@ -15784,46 +15722,42 @@
     </row>
     <row r="119">
       <c r="A119" t="s" s="2">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="B119" t="s" s="2">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="C119" s="2"/>
       <c r="D119" t="s" s="2">
-        <v>286</v>
+        <v>80</v>
       </c>
       <c r="E119" s="2"/>
       <c r="F119" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G119" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="H119" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I119" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="J119" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="K119" t="s" s="2">
-        <v>109</v>
+        <v>254</v>
       </c>
       <c r="L119" t="s" s="2">
-        <v>287</v>
+        <v>623</v>
       </c>
       <c r="M119" t="s" s="2">
-        <v>288</v>
-      </c>
-      <c r="N119" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="O119" t="s" s="2">
-        <v>205</v>
-      </c>
+        <v>624</v>
+      </c>
+      <c r="N119" s="2"/>
+      <c r="O119" s="2"/>
       <c r="P119" t="s" s="2">
         <v>80</v>
       </c>
@@ -15871,25 +15805,25 @@
         <v>80</v>
       </c>
       <c r="AF119" t="s" s="2">
-        <v>289</v>
+        <v>622</v>
       </c>
       <c r="AG119" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH119" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AI119" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ119" t="s" s="2">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="AK119" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL119" t="s" s="2">
-        <v>191</v>
+        <v>420</v>
       </c>
       <c r="AM119" t="s" s="2">
         <v>80</v>
@@ -15911,7 +15845,7 @@
       </c>
       <c r="E120" s="2"/>
       <c r="F120" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="G120" t="s" s="2">
         <v>88</v>
@@ -15926,13 +15860,13 @@
         <v>80</v>
       </c>
       <c r="K120" t="s" s="2">
+        <v>261</v>
+      </c>
+      <c r="L120" t="s" s="2">
         <v>626</v>
       </c>
-      <c r="L120" t="s" s="2">
+      <c r="M120" t="s" s="2">
         <v>627</v>
-      </c>
-      <c r="M120" t="s" s="2">
-        <v>628</v>
       </c>
       <c r="N120" s="2"/>
       <c r="O120" s="2"/>
@@ -15986,7 +15920,7 @@
         <v>625</v>
       </c>
       <c r="AG120" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="AH120" t="s" s="2">
         <v>88</v>
@@ -15998,24 +15932,24 @@
         <v>100</v>
       </c>
       <c r="AK120" t="s" s="2">
+        <v>426</v>
+      </c>
+      <c r="AL120" t="s" s="2">
+        <v>628</v>
+      </c>
+      <c r="AM120" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN120" t="s" s="2">
         <v>629</v>
-      </c>
-      <c r="AL120" t="s" s="2">
-        <v>427</v>
-      </c>
-      <c r="AM120" t="s" s="2">
-        <v>630</v>
-      </c>
-      <c r="AN120" t="s" s="2">
-        <v>631</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="s" s="2">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="B121" t="s" s="2">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="C121" s="2"/>
       <c r="D121" t="s" s="2">
@@ -16038,16 +15972,16 @@
         <v>80</v>
       </c>
       <c r="K121" t="s" s="2">
-        <v>168</v>
+        <v>631</v>
       </c>
       <c r="L121" t="s" s="2">
+        <v>632</v>
+      </c>
+      <c r="M121" t="s" s="2">
         <v>633</v>
       </c>
-      <c r="M121" t="s" s="2">
+      <c r="N121" t="s" s="2">
         <v>634</v>
-      </c>
-      <c r="N121" t="s" s="2">
-        <v>635</v>
       </c>
       <c r="O121" s="2"/>
       <c r="P121" t="s" s="2">
@@ -16073,13 +16007,13 @@
         <v>80</v>
       </c>
       <c r="X121" t="s" s="2">
-        <v>222</v>
+        <v>80</v>
       </c>
       <c r="Y121" t="s" s="2">
-        <v>636</v>
+        <v>80</v>
       </c>
       <c r="Z121" t="s" s="2">
-        <v>637</v>
+        <v>80</v>
       </c>
       <c r="AA121" t="s" s="2">
         <v>80</v>
@@ -16097,7 +16031,7 @@
         <v>80</v>
       </c>
       <c r="AF121" t="s" s="2">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="AG121" t="s" s="2">
         <v>78</v>
@@ -16112,465 +16046,15 @@
         <v>100</v>
       </c>
       <c r="AK121" t="s" s="2">
-        <v>80</v>
+        <v>635</v>
       </c>
       <c r="AL121" t="s" s="2">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="AM121" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN121" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="s" s="2">
-        <v>639</v>
-      </c>
-      <c r="B122" t="s" s="2">
-        <v>639</v>
-      </c>
-      <c r="C122" s="2"/>
-      <c r="D122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="E122" s="2"/>
-      <c r="F122" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G122" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="H122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="I122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="K122" t="s" s="2">
-        <v>228</v>
-      </c>
-      <c r="L122" t="s" s="2">
-        <v>640</v>
-      </c>
-      <c r="M122" t="s" s="2">
-        <v>641</v>
-      </c>
-      <c r="N122" t="s" s="2">
-        <v>642</v>
-      </c>
-      <c r="O122" s="2"/>
-      <c r="P122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q122" s="2"/>
-      <c r="R122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X122" t="s" s="2">
-        <v>158</v>
-      </c>
-      <c r="Y122" s="2"/>
-      <c r="Z122" t="s" s="2">
-        <v>643</v>
-      </c>
-      <c r="AA122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF122" t="s" s="2">
-        <v>639</v>
-      </c>
-      <c r="AG122" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH122" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="AI122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AJ122" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="AK122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM122" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN122" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="s" s="2">
-        <v>644</v>
-      </c>
-      <c r="B123" t="s" s="2">
-        <v>644</v>
-      </c>
-      <c r="C123" s="2"/>
-      <c r="D123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="E123" s="2"/>
-      <c r="F123" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G123" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="H123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="I123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="K123" t="s" s="2">
-        <v>254</v>
-      </c>
-      <c r="L123" t="s" s="2">
-        <v>645</v>
-      </c>
-      <c r="M123" t="s" s="2">
-        <v>646</v>
-      </c>
-      <c r="N123" s="2"/>
-      <c r="O123" s="2"/>
-      <c r="P123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q123" s="2"/>
-      <c r="R123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Z123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AA123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF123" t="s" s="2">
-        <v>644</v>
-      </c>
-      <c r="AG123" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH123" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="AI123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AJ123" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="AK123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL123" t="s" s="2">
-        <v>420</v>
-      </c>
-      <c r="AM123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN123" t="s" s="2">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="s" s="2">
-        <v>647</v>
-      </c>
-      <c r="B124" t="s" s="2">
-        <v>647</v>
-      </c>
-      <c r="C124" s="2"/>
-      <c r="D124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="E124" s="2"/>
-      <c r="F124" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G124" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="H124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="I124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="K124" t="s" s="2">
-        <v>261</v>
-      </c>
-      <c r="L124" t="s" s="2">
-        <v>648</v>
-      </c>
-      <c r="M124" t="s" s="2">
-        <v>649</v>
-      </c>
-      <c r="N124" s="2"/>
-      <c r="O124" s="2"/>
-      <c r="P124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q124" s="2"/>
-      <c r="R124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Z124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AA124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF124" t="s" s="2">
-        <v>647</v>
-      </c>
-      <c r="AG124" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH124" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="AI124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AJ124" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="AK124" t="s" s="2">
-        <v>426</v>
-      </c>
-      <c r="AL124" t="s" s="2">
-        <v>650</v>
-      </c>
-      <c r="AM124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN124" t="s" s="2">
-        <v>651</v>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="s" s="2">
-        <v>652</v>
-      </c>
-      <c r="B125" t="s" s="2">
-        <v>652</v>
-      </c>
-      <c r="C125" s="2"/>
-      <c r="D125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="E125" s="2"/>
-      <c r="F125" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G125" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="H125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="I125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="K125" t="s" s="2">
-        <v>653</v>
-      </c>
-      <c r="L125" t="s" s="2">
-        <v>654</v>
-      </c>
-      <c r="M125" t="s" s="2">
-        <v>655</v>
-      </c>
-      <c r="N125" t="s" s="2">
-        <v>656</v>
-      </c>
-      <c r="O125" s="2"/>
-      <c r="P125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q125" s="2"/>
-      <c r="R125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Z125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AA125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF125" t="s" s="2">
-        <v>652</v>
-      </c>
-      <c r="AG125" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH125" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="AI125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AJ125" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="AK125" t="s" s="2">
-        <v>657</v>
-      </c>
-      <c r="AL125" t="s" s="2">
-        <v>658</v>
-      </c>
-      <c r="AM125" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN125" t="s" s="2">
         <v>80</v>
       </c>
     </row>

</xml_diff>